<commit_message>
add logo and deploy on render
</commit_message>
<xml_diff>
--- a/Backend/icnome_details.xlsx
+++ b/Backend/icnome_details.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,10 +415,10 @@
         <v>salary</v>
       </c>
       <c r="B2">
-        <v>230</v>
+        <v>5000</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-02-24</v>
+        <v>2026-02-23</v>
       </c>
     </row>
     <row r="3">
@@ -426,114 +426,15 @@
         <v>salary</v>
       </c>
       <c r="B3">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-02-24</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Gift</v>
-      </c>
-      <c r="B4">
-        <v>230</v>
-      </c>
-      <c r="C4" t="str">
         <v>2026-02-23</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>freelanc</v>
-      </c>
-      <c r="B5">
-        <v>100</v>
-      </c>
-      <c r="C5" t="str">
-        <v>2026-02-23</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>course</v>
-      </c>
-      <c r="B6">
-        <v>30</v>
-      </c>
-      <c r="C6" t="str">
-        <v>2026-02-19</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>salary</v>
-      </c>
-      <c r="B7">
-        <v>5000</v>
-      </c>
-      <c r="C7" t="str">
-        <v>2026-02-19</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Course</v>
-      </c>
-      <c r="B8">
-        <v>25</v>
-      </c>
-      <c r="C8" t="str">
-        <v>2026-02-18</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Salary</v>
-      </c>
-      <c r="B9">
-        <v>20</v>
-      </c>
-      <c r="C9" t="str">
-        <v>2026-02-17</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>tcs</v>
-      </c>
-      <c r="B10">
-        <v>340</v>
-      </c>
-      <c r="C10" t="str">
-        <v>2026-02-17</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>salary</v>
-      </c>
-      <c r="B11">
-        <v>100</v>
-      </c>
-      <c r="C11" t="str">
-        <v>2026-02-17</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Freelancer</v>
-      </c>
-      <c r="B12">
-        <v>150</v>
-      </c>
-      <c r="C12" t="str">
-        <v>2026-02-16</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>